<commit_message>
updated the endpoint for player list
</commit_message>
<xml_diff>
--- a/players.xlsx
+++ b/players.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="233">
   <si>
     <t>Sl.No</t>
   </si>
@@ -44,6 +44,9 @@
     <t>id</t>
   </si>
   <si>
+    <t>category</t>
+  </si>
+  <si>
     <t xml:space="preserve">Chetan kumar </t>
   </si>
   <si>
@@ -53,6 +56,9 @@
     <t>9620250934</t>
   </si>
   <si>
+    <t>A+</t>
+  </si>
+  <si>
     <t xml:space="preserve">Azeez Ur Rahman </t>
   </si>
   <si>
@@ -116,6 +122,9 @@
     <t>9743474289</t>
   </si>
   <si>
+    <t>A</t>
+  </si>
+  <si>
     <t>Mohammed noor afnan</t>
   </si>
   <si>
@@ -179,6 +188,9 @@
     <t>9677325317</t>
   </si>
   <si>
+    <t>B+</t>
+  </si>
+  <si>
     <t>Vijay</t>
   </si>
   <si>
@@ -242,6 +254,9 @@
     <t>9538015554</t>
   </si>
   <si>
+    <t>B</t>
+  </si>
+  <si>
     <t>STEPHEN</t>
   </si>
   <si>
@@ -305,6 +320,9 @@
     <t>8105350075</t>
   </si>
   <si>
+    <t>c+</t>
+  </si>
+  <si>
     <t xml:space="preserve">AHMED ZUBAIR </t>
   </si>
   <si>
@@ -359,6 +377,9 @@
     <t>9108280746</t>
   </si>
   <si>
+    <t>c</t>
+  </si>
+  <si>
     <t>SYED ZAINUL ABIDDIN</t>
   </si>
   <si>
@@ -413,6 +434,9 @@
     <t>8130498848</t>
   </si>
   <si>
+    <t>D+</t>
+  </si>
+  <si>
     <t xml:space="preserve">ACHINTHYA </t>
   </si>
   <si>
@@ -467,6 +491,9 @@
     <t>8951892520</t>
   </si>
   <si>
+    <t>D</t>
+  </si>
+  <si>
     <t>NADEEM KHAN</t>
   </si>
   <si>
@@ -521,6 +548,9 @@
     <t>9844959285</t>
   </si>
   <si>
+    <t>E+</t>
+  </si>
+  <si>
     <t xml:space="preserve">Nawaz pasha </t>
   </si>
   <si>
@@ -584,6 +614,9 @@
     <t>8553328785</t>
   </si>
   <si>
+    <t>E</t>
+  </si>
+  <si>
     <t>AFTAB AHMED</t>
   </si>
   <si>
@@ -636,6 +669,9 @@
   </si>
   <si>
     <t>9620525705</t>
+  </si>
+  <si>
+    <t>W</t>
   </si>
   <si>
     <t>Raghu R</t>
@@ -702,7 +738,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -724,13 +760,6 @@
       <color theme="10"/>
       <name val="Calibri"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -1198,149 +1227,149 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1704,17 +1733,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E73"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelCol="4"/>
+  <dimension ref="A1:F73"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="21.1" customWidth="1"/>
     <col min="2" max="2" width="32.2" customWidth="1"/>
     <col min="3" max="3" width="98.2" customWidth="1"/>
     <col min="4" max="4" width="30" customWidth="1"/>
     <col min="5" max="5" width="35.6" customWidth="1"/>
+    <col min="6" max="6" width="25.1363636363636" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1730,1229 +1760,1448 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E2" s="4">
         <v>2265635</v>
       </c>
-    </row>
-    <row r="3" spans="1:5">
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E3" s="4">
         <v>2330581</v>
       </c>
-    </row>
-    <row r="4" spans="1:5">
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E4" s="4">
         <v>14228489</v>
       </c>
-    </row>
-    <row r="5" spans="1:5">
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E5" s="4">
         <v>1392508</v>
       </c>
-    </row>
-    <row r="6" spans="1:5">
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D6" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E6" s="4">
         <v>1770010</v>
       </c>
-    </row>
-    <row r="7" spans="1:5">
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E7" s="4">
         <v>6793605</v>
       </c>
-    </row>
-    <row r="8" spans="1:5">
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D8" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E8" s="4">
         <v>11028778</v>
       </c>
-    </row>
-    <row r="9" spans="1:5">
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E9" s="4">
         <v>196670</v>
       </c>
-    </row>
-    <row r="10" spans="1:5">
+      <c r="F9" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="D10" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E10" s="4">
         <v>2265213</v>
       </c>
-    </row>
-    <row r="11" spans="1:5">
+      <c r="F10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D11" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="E11" s="4">
         <v>6352344</v>
       </c>
-    </row>
-    <row r="12" spans="1:5">
+      <c r="F11" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D12" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E12" s="4">
         <v>7329730</v>
       </c>
-    </row>
-    <row r="13" spans="1:5">
+      <c r="F12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D13" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E13" s="4">
         <v>914349</v>
       </c>
-    </row>
-    <row r="14" spans="1:5">
+      <c r="F13" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D14" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="E14" s="4">
         <v>2116796</v>
       </c>
-    </row>
-    <row r="15" spans="1:5">
+      <c r="F14" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D15" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E15" s="4">
         <v>2593031</v>
       </c>
-    </row>
-    <row r="16" spans="1:5">
+      <c r="F15" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="D16" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E16" s="4">
         <v>11689699</v>
       </c>
-    </row>
-    <row r="17" spans="1:5">
+      <c r="F16" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
       <c r="A17">
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="D17" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="E17" s="4">
         <v>3689437</v>
       </c>
-    </row>
-    <row r="18" spans="1:5">
+      <c r="F17" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="D18" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="E18" s="4">
         <v>11194603</v>
       </c>
-    </row>
-    <row r="19" spans="1:5">
+      <c r="F18" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D19" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="E19" s="4">
         <v>3055708</v>
       </c>
-    </row>
-    <row r="20" spans="1:5">
+      <c r="F19" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="D20" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="E20" s="4">
         <v>13515484</v>
       </c>
-    </row>
-    <row r="21" spans="1:5">
+      <c r="F20" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
       <c r="A21">
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D21" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E21" s="4">
         <v>10068046</v>
       </c>
-    </row>
-    <row r="22" spans="1:5">
+      <c r="F21" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
       <c r="A22">
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D22" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="E22" s="4">
         <v>3758036</v>
       </c>
-    </row>
-    <row r="23" spans="1:5">
+      <c r="F22" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
       <c r="A23">
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="D23" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="E23" s="4">
         <v>20685806</v>
       </c>
-    </row>
-    <row r="24" spans="1:5">
+      <c r="F23" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
       <c r="A24">
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="D24" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="E24" s="4">
         <v>7009059</v>
       </c>
-    </row>
-    <row r="25" spans="1:5">
+      <c r="F24" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D25" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="E25" s="4">
         <v>5925631</v>
       </c>
-    </row>
-    <row r="26" spans="1:5">
+      <c r="F25" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
       <c r="A26">
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="D26" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E26" s="4">
         <v>10054506</v>
       </c>
-    </row>
-    <row r="27" spans="1:5">
+      <c r="F26" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
       <c r="A27">
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="D27" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="E27" s="4">
         <v>1206842</v>
       </c>
-    </row>
-    <row r="28" spans="1:5">
+      <c r="F27" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
       <c r="A28">
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="D28" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="E28" s="4">
         <v>6049307</v>
       </c>
-    </row>
-    <row r="29" spans="1:5">
+      <c r="F28" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
       <c r="A29">
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="D29" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="E29" s="4">
         <v>658382</v>
       </c>
-    </row>
-    <row r="30" spans="1:5">
+      <c r="F29" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
       <c r="A30">
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="D30" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="E30" s="4">
         <v>3589804</v>
       </c>
-    </row>
-    <row r="31" spans="1:5">
+      <c r="F30" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
       <c r="A31">
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="D31" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="E31" s="4">
         <v>511404</v>
       </c>
-    </row>
-    <row r="32" spans="1:5">
+      <c r="F31" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
       <c r="A32">
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D32" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="E32" s="4">
         <v>16312321</v>
       </c>
-    </row>
-    <row r="33" spans="1:5">
+      <c r="F32" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
       <c r="A33">
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D33" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="E33" s="4">
         <v>2625600</v>
       </c>
-    </row>
-    <row r="34" spans="1:5">
+      <c r="F33" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
       <c r="A34">
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="D34" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="E34" s="4">
         <v>134340</v>
       </c>
-    </row>
-    <row r="35" spans="1:5">
+      <c r="F34" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
       <c r="A35">
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="D35" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="E35" s="4">
         <v>30444707</v>
       </c>
-    </row>
-    <row r="36" spans="1:5">
+      <c r="F35" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
       <c r="A36">
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="D36" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="E36" s="4">
         <v>15268543</v>
       </c>
-    </row>
-    <row r="37" spans="1:5">
+      <c r="F36" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
       <c r="A37">
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="D37" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="E37" s="4">
         <v>7330144</v>
       </c>
-    </row>
-    <row r="38" spans="1:5">
+      <c r="F37" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6">
       <c r="A38">
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="D38" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="E38" s="4">
         <v>6190456</v>
       </c>
-    </row>
-    <row r="39" spans="1:5">
+      <c r="F38" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
       <c r="A39">
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="D39" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="E39" s="4">
         <v>2775365</v>
       </c>
-    </row>
-    <row r="40" spans="1:5">
+      <c r="F39" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6">
       <c r="A40">
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="D40" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="E40" s="4">
         <v>8910543</v>
       </c>
-    </row>
-    <row r="41" spans="1:5">
+      <c r="F40" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6">
       <c r="A41">
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="D41" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="E41" s="4">
         <v>8167969</v>
       </c>
-    </row>
-    <row r="42" spans="1:5">
+      <c r="F41" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
       <c r="A42">
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="D42" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="E42" s="4">
         <v>2063329</v>
       </c>
-    </row>
-    <row r="43" spans="1:5">
+      <c r="F42" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6">
       <c r="A43">
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="D43" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="E43" s="4">
         <v>2874663</v>
       </c>
-    </row>
-    <row r="44" spans="1:5">
+      <c r="F43" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6">
       <c r="A44">
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="D44" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E44" s="4">
         <v>1108113</v>
       </c>
-    </row>
-    <row r="45" spans="1:5">
+      <c r="F44" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6">
       <c r="A45">
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="D45" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="E45" s="4">
         <v>17211485</v>
       </c>
-    </row>
-    <row r="46" spans="1:5">
+      <c r="F45" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6">
       <c r="A46">
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="D46" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="E46" s="4">
         <v>12246396</v>
       </c>
-    </row>
-    <row r="47" spans="1:5">
+      <c r="F46" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6">
       <c r="A47">
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="D47" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="E47" s="4">
         <v>774977</v>
       </c>
-    </row>
-    <row r="48" spans="1:5">
+      <c r="F47" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6">
       <c r="A48">
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="D48" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="E48" s="4">
         <v>6076059</v>
       </c>
-    </row>
-    <row r="49" spans="1:5">
+      <c r="F48" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6">
       <c r="A49">
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>146</v>
+        <v>155</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>147</v>
+        <v>156</v>
       </c>
       <c r="D49" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="E49" s="4">
         <v>2292736</v>
       </c>
-    </row>
-    <row r="50" spans="1:5">
+      <c r="F49" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6">
       <c r="A50">
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>149</v>
+        <v>158</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="D50" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="E50" s="4">
         <v>6315988</v>
       </c>
-    </row>
-    <row r="51" spans="1:5">
+      <c r="F50" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6">
       <c r="A51">
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="D51" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="E51" s="4">
         <v>972616</v>
       </c>
-    </row>
-    <row r="52" spans="1:5">
+      <c r="F51" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6">
       <c r="A52">
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="D52" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="E52" s="4">
         <v>3302781</v>
       </c>
-    </row>
-    <row r="53" spans="1:5">
+      <c r="F52" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6">
       <c r="A53">
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>158</v>
+        <v>167</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="D53" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
       <c r="E53" s="4">
         <v>11804862</v>
       </c>
-    </row>
-    <row r="54" spans="1:5">
+      <c r="F53" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6">
       <c r="A54">
         <v>53</v>
       </c>
       <c r="B54" t="s">
-        <v>161</v>
+        <v>170</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>162</v>
+        <v>171</v>
       </c>
       <c r="D54" t="s">
-        <v>163</v>
+        <v>172</v>
       </c>
       <c r="E54" s="4">
         <v>11760152</v>
       </c>
-    </row>
-    <row r="55" spans="1:5">
+      <c r="F54" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6">
       <c r="A55">
         <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>164</v>
+        <v>174</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="D55" t="s">
-        <v>166</v>
+        <v>176</v>
       </c>
       <c r="E55" s="4">
         <v>16029309</v>
       </c>
-    </row>
-    <row r="56" spans="1:5">
+      <c r="F55" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6">
       <c r="A56">
         <v>55</v>
       </c>
       <c r="B56" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="D56" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="E56" s="4">
         <v>6517797</v>
       </c>
-    </row>
-    <row r="57" spans="1:5">
+      <c r="F56" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6">
       <c r="A57">
         <v>56</v>
       </c>
       <c r="B57" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
       <c r="D57" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
       <c r="E57" s="4">
         <v>2265640</v>
       </c>
-    </row>
-    <row r="58" spans="1:5">
+      <c r="F57" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6">
       <c r="A58">
         <v>57</v>
       </c>
       <c r="B58" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
       <c r="D58" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
       <c r="E58" s="4">
         <v>1077553</v>
       </c>
-    </row>
-    <row r="59" spans="1:5">
+      <c r="F58" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6">
       <c r="A59">
         <v>58</v>
       </c>
       <c r="B59" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>177</v>
+        <v>187</v>
       </c>
       <c r="D59" t="s">
-        <v>178</v>
+        <v>188</v>
       </c>
       <c r="E59" s="4">
         <v>306601</v>
       </c>
-    </row>
-    <row r="60" spans="1:5">
+      <c r="F59" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6">
       <c r="A60">
         <v>59</v>
       </c>
       <c r="B60" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="D60" t="s">
-        <v>181</v>
+        <v>191</v>
       </c>
       <c r="E60" s="4">
         <v>25215761</v>
       </c>
-    </row>
-    <row r="61" spans="1:5">
+      <c r="F60" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6">
       <c r="A61">
         <v>60</v>
       </c>
       <c r="B61" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
       <c r="D61" t="s">
-        <v>184</v>
+        <v>194</v>
       </c>
       <c r="E61" s="4">
         <v>1108115</v>
       </c>
-    </row>
-    <row r="62" spans="1:5">
+      <c r="F61" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6">
       <c r="A62">
         <v>61</v>
       </c>
       <c r="B62" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>186</v>
+        <v>197</v>
       </c>
       <c r="D62" t="s">
-        <v>187</v>
+        <v>198</v>
       </c>
       <c r="E62" s="4">
         <v>13356710</v>
       </c>
-    </row>
-    <row r="63" spans="1:5">
+      <c r="F62" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6">
       <c r="A63">
         <v>62</v>
       </c>
       <c r="B63" t="s">
-        <v>188</v>
+        <v>199</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>189</v>
+        <v>200</v>
       </c>
       <c r="D63" t="s">
-        <v>190</v>
+        <v>201</v>
       </c>
       <c r="E63" s="4">
         <v>1388686</v>
       </c>
-    </row>
-    <row r="64" spans="1:5">
+      <c r="F63" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6">
       <c r="A64">
         <v>63</v>
       </c>
       <c r="B64" t="s">
-        <v>191</v>
+        <v>202</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="D64" t="s">
-        <v>193</v>
+        <v>204</v>
       </c>
       <c r="E64" s="4">
         <v>8849263</v>
       </c>
-    </row>
-    <row r="65" spans="1:5">
+      <c r="F64" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6">
       <c r="A65">
         <v>64</v>
       </c>
       <c r="B65" t="s">
-        <v>194</v>
+        <v>205</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>195</v>
+        <v>206</v>
       </c>
       <c r="D65" t="s">
-        <v>196</v>
+        <v>207</v>
       </c>
       <c r="E65" s="4">
         <v>3758867</v>
       </c>
-    </row>
-    <row r="66" spans="1:5">
+      <c r="F65" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6">
       <c r="A66">
         <v>65</v>
       </c>
       <c r="B66" t="s">
-        <v>197</v>
+        <v>208</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>198</v>
+        <v>209</v>
       </c>
       <c r="D66" t="s">
-        <v>199</v>
+        <v>210</v>
       </c>
       <c r="E66" s="4">
         <v>3754330</v>
       </c>
-    </row>
-    <row r="67" spans="1:5">
+      <c r="F66" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6">
       <c r="A67">
         <v>66</v>
       </c>
       <c r="B67" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>201</v>
+        <v>212</v>
       </c>
       <c r="D67" t="s">
-        <v>202</v>
+        <v>213</v>
       </c>
       <c r="E67" s="4">
         <v>10950858</v>
       </c>
-    </row>
-    <row r="68" spans="1:5">
+      <c r="F67" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6">
       <c r="A68">
         <v>67</v>
       </c>
       <c r="B68" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>204</v>
+        <v>216</v>
       </c>
       <c r="D68" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="E68" s="4">
         <v>43564284</v>
       </c>
-    </row>
-    <row r="69" spans="1:5">
+      <c r="F68" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6">
       <c r="A69">
         <v>68</v>
       </c>
       <c r="B69" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>207</v>
+        <v>219</v>
       </c>
       <c r="D69" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
       <c r="E69" s="4">
         <v>1764668</v>
       </c>
-    </row>
-    <row r="70" spans="1:5">
+      <c r="F69" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6">
       <c r="A70">
         <v>69</v>
       </c>
       <c r="B70" t="s">
-        <v>209</v>
+        <v>221</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="D70" t="s">
-        <v>211</v>
+        <v>223</v>
       </c>
       <c r="E70" s="4">
         <v>387238</v>
       </c>
-    </row>
-    <row r="71" spans="1:5">
+      <c r="F70" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6">
       <c r="A71">
         <v>70</v>
       </c>
       <c r="B71" t="s">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="D71" t="s">
-        <v>214</v>
+        <v>226</v>
       </c>
       <c r="E71" s="4">
         <v>5925592</v>
       </c>
-    </row>
-    <row r="72" spans="1:5">
+      <c r="F71" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6">
       <c r="A72">
         <v>71</v>
       </c>
       <c r="B72" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>216</v>
+        <v>228</v>
       </c>
       <c r="D72" t="s">
-        <v>217</v>
+        <v>229</v>
       </c>
       <c r="E72" s="4">
         <v>12610609</v>
       </c>
-    </row>
-    <row r="73" spans="1:5">
+      <c r="F72" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6">
       <c r="A73">
         <v>72</v>
       </c>
       <c r="B73" t="s">
-        <v>218</v>
+        <v>230</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>219</v>
+        <v>231</v>
       </c>
       <c r="D73" t="s">
-        <v>220</v>
+        <v>232</v>
       </c>
       <c r="E73" s="4">
         <v>16929490</v>
+      </c>
+      <c r="F73" t="s">
+        <v>214</v>
       </c>
     </row>
   </sheetData>

</xml_diff>